<commit_message>
log previous best prices
</commit_message>
<xml_diff>
--- a/project_files/prixEpicerie.xlsx
+++ b/project_files/prixEpicerie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dalto\OneDrive\Documents\Ecole\Programmation1\Team_Rosemarie_and_Leo\project_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E223B1D3-B6FE-4AD6-B06D-B72059795315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AF452E-E2F9-46FD-A27B-BE276A27C413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{2198D66A-2FBF-4C5F-A307-23CE27175DD6}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
   <si>
     <t>Apple</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>juice</t>
+  </si>
+  <si>
+    <t>eggs</t>
   </si>
 </sst>
 </file>
@@ -481,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D0CAF0-E220-42F4-9499-7F81EB90A030}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -505,7 +508,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="3">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -538,6 +541,14 @@
       </c>
       <c r="B7" s="3">
         <v>1.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3">
+        <v>1.3</v>
       </c>
     </row>
   </sheetData>
@@ -548,7 +559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C57A07B-F668-49AB-9E14-5DC649963E41}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -607,6 +618,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
lol des changement de shit dans mon pc ont regle des probleme
</commit_message>
<xml_diff>
--- a/project_files/prixEpicerie.xlsx
+++ b/project_files/prixEpicerie.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dalto\OneDrive\Documents\Ecole\Programmation1\Team_Rosemarie_and_Leo\project_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4e83fdffc868d823/projet_prog/Team_Rosemarie_and_Leo/project_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AF452E-E2F9-46FD-A27B-BE276A27C413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{83AF452E-E2F9-46FD-A27B-BE276A27C413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52BEC1D5-61A6-4EFE-92E1-79C1C19A441E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{2198D66A-2FBF-4C5F-A307-23CE27175DD6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2198D66A-2FBF-4C5F-A307-23CE27175DD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Metro" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="10">
   <si>
     <t>Apple</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>eggs</t>
+  </si>
+  <si>
+    <t>laitue</t>
   </si>
 </sst>
 </file>
@@ -71,7 +74,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -142,13 +145,13 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Monétaire" xfId="1" builtinId="4"/>
@@ -484,10 +487,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D0CAF0-E220-42F4-9499-7F81EB90A030}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -495,7 +498,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -503,7 +506,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -511,7 +514,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -519,7 +522,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -527,7 +530,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -535,7 +538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -543,12 +546,20 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="3">
         <v>1.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -559,10 +570,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C57A07B-F668-49AB-9E14-5DC649963E41}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -570,7 +581,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -578,7 +589,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -586,7 +597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -594,7 +605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -602,7 +613,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -610,7 +621,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -618,12 +629,20 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="3">
         <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>